<commit_message>
feat: pengguna memilih akun master sendiri + urutannya
- Sheet baru AkunPengguna (id, user_id, akun_id, urutan, audit)
- GET/PUT /api/akun/pilihan; GET /api/akun memakai pilihan & urutan pengguna
- Pengguna tanpa pilihan = semua akun aktif (pengguna lama)
- Akun tidak dipilih ditolak di transaksi, langganan, tarik tabungan, saldo awal
- Akun bersaldo ≠ 0 di periode aktif tidak bisa dilepas
- Ringkasan & dashboard urut menurut pengguna
- Pengaturan → Akun saya: centang akun + atur urutan dengan drag & drop (@dnd-kit)

Co-Authored-By: WOZCODE <contact@withwoz.com>
</commit_message>
<xml_diff>
--- a/template/Saku_Template.xlsx
+++ b/template/Saku_Template.xlsx
@@ -7,13 +7,14 @@
     <sheet sheetId="1" name="Panduan" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Pengguna" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Akun" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Kategori" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Periode" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="SaldoAwal" state="visible" r:id="rId9"/>
-    <sheet sheetId="7" name="Transaksi" state="visible" r:id="rId10"/>
-    <sheet sheetId="8" name="Berulang" state="visible" r:id="rId11"/>
-    <sheet sheetId="9" name="BerulangLewati" state="visible" r:id="rId12"/>
-    <sheet sheetId="10" name="Tabungan" state="visible" r:id="rId13"/>
+    <sheet sheetId="4" name="AkunPengguna" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Kategori" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="Periode" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="SaldoAwal" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="Transaksi" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="Berulang" state="visible" r:id="rId12"/>
+    <sheet sheetId="10" name="BerulangLewati" state="visible" r:id="rId13"/>
+    <sheet sheetId="11" name="Tabungan" state="visible" r:id="rId14"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -28,6 +29,58 @@
     <comment ref="A1" authorId="0">
       <text>
         <r>
+          <t>RL-xxxxxxxx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0">
+      <text>
+        <r>
+          <t>yyyy-MM. Unik per (berulang_id, bulan).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0">
+      <text>
+        <r>
+          <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0">
+      <text>
+        <r>
+          <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0">
+      <text>
+        <r>
+          <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0">
+      <text>
+        <r>
+          <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments11.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Author</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0">
+      <text>
+        <r>
           <t>TB-xxxxxxxx</t>
         </r>
       </text>
@@ -251,31 +304,10 @@
     <author>Author</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0">
-      <text>
-        <r>
-          <t>KT-xxxxxxxx. Master bersama semua pengguna, hanya admin yang mengubah.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0">
-      <text>
-        <r>
-          <t>1–40 karakter, unik per tipe di antara kategori aktif.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0">
-      <text>
-        <r>
-          <t>masuk / keluar</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0">
-      <text>
-        <r>
-          <t>Kosong, BIAYA_ADMIN (keluar), atau TARIK_TABUNGAN (masuk). Kategori sistem tidak bisa dinonaktifkan.</t>
+    <comment ref="E1" authorId="0">
+      <text>
+        <r>
+          <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
         </r>
       </text>
     </comment>
@@ -294,13 +326,6 @@
       </text>
     </comment>
     <comment ref="H1" authorId="0">
-      <text>
-        <r>
-          <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0">
       <text>
         <r>
           <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
@@ -320,21 +345,35 @@
     <comment ref="A1" authorId="0">
       <text>
         <r>
-          <t>PR-xxxxxxxx</t>
+          <t>KT-xxxxxxxx. Master bersama semua pengguna, hanya admin yang mengubah.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0">
+      <text>
+        <r>
+          <t>1–40 karakter, unik per tipe di antara kategori aktif.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0">
+      <text>
+        <r>
+          <t>masuk / keluar</t>
         </r>
       </text>
     </comment>
     <comment ref="D1" authorId="0">
       <text>
         <r>
-          <t>yyyy-MM-dd</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0">
-      <text>
-        <r>
-          <t>Kosong = periode aktif. Maksimal 1 aktif per pengguna.</t>
+          <t>Kosong, BIAYA_ADMIN (keluar), atau TARIK_TABUNGAN (masuk). Kategori sistem tidak bisa dinonaktifkan.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0">
+      <text>
+        <r>
+          <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
         </r>
       </text>
     </comment>
@@ -353,13 +392,6 @@
       </text>
     </comment>
     <comment ref="I1" authorId="0">
-      <text>
-        <r>
-          <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0">
       <text>
         <r>
           <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
@@ -379,46 +411,46 @@
     <comment ref="A1" authorId="0">
       <text>
         <r>
-          <t>SA-xxxxxxxx</t>
+          <t>PR-xxxxxxxx</t>
         </r>
       </text>
     </comment>
     <comment ref="D1" authorId="0">
       <text>
         <r>
-          <t>Unik per (periode_id, akun_id).</t>
+          <t>yyyy-MM-dd</t>
         </r>
       </text>
     </comment>
     <comment ref="E1" authorId="0">
       <text>
         <r>
-          <t>Angka ≥ 0, tanpa titik.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0">
+          <t>Kosong = periode aktif. Maksimal 1 aktif per pengguna.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0">
       <text>
         <r>
           <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0">
+    <comment ref="H1" authorId="0">
       <text>
         <r>
           <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0">
+    <comment ref="I1" authorId="0">
       <text>
         <r>
           <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0">
+    <comment ref="J1" authorId="0">
       <text>
         <r>
           <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
@@ -438,102 +470,46 @@
     <comment ref="A1" authorId="0">
       <text>
         <r>
-          <t>TR-xxxxxxxx</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0">
-      <text>
-        <r>
-          <t>Ditentukan server dari tanggal.</t>
+          <t>SA-xxxxxxxx</t>
         </r>
       </text>
     </comment>
     <comment ref="D1" authorId="0">
       <text>
         <r>
-          <t>yyyy-MM-dd</t>
+          <t>Unik per (periode_id, akun_id).</t>
         </r>
       </text>
     </comment>
     <comment ref="E1" authorId="0">
       <text>
         <r>
-          <t>keluar / masuk / transfer</t>
+          <t>Angka ≥ 0, tanpa titik.</t>
         </r>
       </text>
     </comment>
     <comment ref="F1" authorId="0">
       <text>
         <r>
-          <t>Sumber (keluar/transfer) atau penerima (masuk).</t>
+          <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
         </r>
       </text>
     </comment>
     <comment ref="G1" authorId="0">
       <text>
         <r>
-          <t>Wajib untuk transfer, kosong untuk lainnya.</t>
+          <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
         </r>
       </text>
     </comment>
     <comment ref="H1" authorId="0">
       <text>
         <r>
-          <t>Wajib untuk keluar/masuk, kosong untuk transfer.</t>
+          <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
         </r>
       </text>
     </comment>
     <comment ref="I1" authorId="0">
-      <text>
-        <r>
-          <t>Angka &gt; 0, tanpa titik.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0">
-      <text>
-        <r>
-          <t>Hanya untuk transfer, selain itu 0.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0">
-      <text>
-        <r>
-          <t>Maks 200 karakter.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="L1" authorId="0">
-      <text>
-        <r>
-          <t>Diisi saat konfirmasi langganan.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M1" authorId="0">
-      <text>
-        <r>
-          <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="N1" authorId="0">
-      <text>
-        <r>
-          <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O1" authorId="0">
-      <text>
-        <r>
-          <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="P1" authorId="0">
       <text>
         <r>
           <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
@@ -553,67 +529,102 @@
     <comment ref="A1" authorId="0">
       <text>
         <r>
-          <t>RB-xxxxxxxx</t>
+          <t>TR-xxxxxxxx</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0">
+      <text>
+        <r>
+          <t>Ditentukan server dari tanggal.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0">
+      <text>
+        <r>
+          <t>yyyy-MM-dd</t>
         </r>
       </text>
     </comment>
     <comment ref="E1" authorId="0">
       <text>
         <r>
-          <t>Kategori keluar yang aktif.</t>
+          <t>keluar / masuk / transfer</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0">
+      <text>
+        <r>
+          <t>Sumber (keluar/transfer) atau penerima (masuk).</t>
         </r>
       </text>
     </comment>
     <comment ref="G1" authorId="0">
       <text>
         <r>
-          <t>1–31. Bulan yang lebih pendek → hari terakhir bulan itu.</t>
+          <t>Wajib untuk transfer, kosong untuk lainnya.</t>
         </r>
       </text>
     </comment>
     <comment ref="H1" authorId="0">
       <text>
         <r>
-          <t>0–15 hari sebelum jatuh tempo, default 3.</t>
+          <t>Wajib untuk keluar/masuk, kosong untuk transfer.</t>
         </r>
       </text>
     </comment>
     <comment ref="I1" authorId="0">
       <text>
         <r>
-          <t>yyyy-MM</t>
+          <t>Angka &gt; 0, tanpa titik.</t>
         </r>
       </text>
     </comment>
     <comment ref="J1" authorId="0">
       <text>
         <r>
-          <t>yyyy-MM. Kosong = tanpa batas.</t>
+          <t>Hanya untuk transfer, selain itu 0.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0">
+      <text>
+        <r>
+          <t>Maks 200 karakter.</t>
         </r>
       </text>
     </comment>
     <comment ref="L1" authorId="0">
       <text>
         <r>
+          <t>Diisi saat konfirmasi langganan.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0">
+      <text>
+        <r>
           <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
         </r>
       </text>
     </comment>
-    <comment ref="M1" authorId="0">
+    <comment ref="N1" authorId="0">
       <text>
         <r>
           <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
         </r>
       </text>
     </comment>
-    <comment ref="N1" authorId="0">
+    <comment ref="O1" authorId="0">
       <text>
         <r>
           <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
         </r>
       </text>
     </comment>
-    <comment ref="O1" authorId="0">
+    <comment ref="P1" authorId="0">
       <text>
         <r>
           <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
@@ -633,39 +644,67 @@
     <comment ref="A1" authorId="0">
       <text>
         <r>
-          <t>RL-xxxxxxxx</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0">
-      <text>
-        <r>
-          <t>yyyy-MM. Unik per (berulang_id, bulan).</t>
+          <t>RB-xxxxxxxx</t>
         </r>
       </text>
     </comment>
     <comment ref="E1" authorId="0">
       <text>
         <r>
+          <t>Kategori keluar yang aktif.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0">
+      <text>
+        <r>
+          <t>1–31. Bulan yang lebih pendek → hari terakhir bulan itu.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0">
+      <text>
+        <r>
+          <t>0–15 hari sebelum jatuh tempo, default 3.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0">
+      <text>
+        <r>
+          <t>yyyy-MM</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0">
+      <text>
+        <r>
+          <t>yyyy-MM. Kosong = tanpa batas.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0">
+      <text>
+        <r>
           <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
         </r>
       </text>
     </comment>
-    <comment ref="F1" authorId="0">
+    <comment ref="M1" authorId="0">
       <text>
         <r>
           <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0">
+    <comment ref="N1" authorId="0">
       <text>
         <r>
           <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0">
+    <comment ref="O1" authorId="0">
       <text>
         <r>
           <t>Diisi otomatis oleh API. Jangan diisi manual.</t>
@@ -677,7 +716,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="114">
   <si>
     <t>Saku</t>
   </si>
@@ -733,7 +772,7 @@
     <t>Sheet</t>
   </si>
   <si>
-    <t>Pengguna · Akun · Kategori · Periode · SaldoAwal · Transaksi · Berulang · BerulangLewati · Tabungan</t>
+    <t>Pengguna · Akun · AkunPengguna · Kategori · Periode · SaldoAwal · Transaksi · Berulang · BerulangLewati · Tabungan</t>
   </si>
   <si>
     <t>Detail setiap kolom ada di catatan (hover) pada header.</t>
@@ -787,7 +826,7 @@
     <t>urutan</t>
   </si>
   <si>
-    <t>AK-nxlfnqu6</t>
+    <t>AK-yecapoqj</t>
   </si>
   <si>
     <t>Bank Jawa Timur</t>
@@ -799,22 +838,22 @@
     <t>SYSTEM</t>
   </si>
   <si>
-    <t>2026-10-30T10:02:58+07:00</t>
-  </si>
-  <si>
-    <t>AK-n63lgyki</t>
+    <t>2026-11-01T14:51:21+07:00</t>
+  </si>
+  <si>
+    <t>AK-oggv435m</t>
   </si>
   <si>
     <t>Bank Negara Indonesia</t>
   </si>
   <si>
-    <t>AK-mdyh7qlx</t>
+    <t>AK-qo6amigc</t>
   </si>
   <si>
     <t>Blu Digital</t>
   </si>
   <si>
-    <t>AK-3kja6p63</t>
+    <t>AK-25nw4qhf</t>
   </si>
   <si>
     <t>GoPay</t>
@@ -823,7 +862,7 @@
     <t>ewallet</t>
   </si>
   <si>
-    <t>AK-gfwkbj3m</t>
+    <t>AK-fj62mtix</t>
   </si>
   <si>
     <t>Cash</t>
@@ -832,13 +871,19 @@
     <t>cash</t>
   </si>
   <si>
+    <t>user_id</t>
+  </si>
+  <si>
+    <t>akun_id</t>
+  </si>
+  <si>
     <t>tipe</t>
   </si>
   <si>
     <t>kode_sistem</t>
   </si>
   <si>
-    <t>KT-66ot76ay</t>
+    <t>KT-yn4mnabf</t>
   </si>
   <si>
     <t>Bonus</t>
@@ -847,37 +892,37 @@
     <t>masuk</t>
   </si>
   <si>
-    <t>KT-xoovhiak</t>
+    <t>KT-di7tcgil</t>
   </si>
   <si>
     <t>Freelance</t>
   </si>
   <si>
-    <t>KT-ueqq2ypl</t>
+    <t>KT-ax6t3xxb</t>
   </si>
   <si>
     <t>Refund</t>
   </si>
   <si>
-    <t>KT-z3aigem6</t>
+    <t>KT-krmncda3</t>
   </si>
   <si>
     <t>Pemberian</t>
   </si>
   <si>
-    <t>KT-k23kubyk</t>
+    <t>KT-ztm4nff7</t>
   </si>
   <si>
     <t>Bunga Bank</t>
   </si>
   <si>
-    <t>KT-relpecwj</t>
+    <t>KT-bbtstagl</t>
   </si>
   <si>
     <t>Lainnya</t>
   </si>
   <si>
-    <t>KT-aer7mwou</t>
+    <t>KT-eiray24e</t>
   </si>
   <si>
     <t>Tarik Tabungan</t>
@@ -886,7 +931,7 @@
     <t>TARIK_TABUNGAN</t>
   </si>
   <si>
-    <t>KT-iyy3kler</t>
+    <t>KT-plv63ner</t>
   </si>
   <si>
     <t>Makan &amp; Minum</t>
@@ -895,61 +940,61 @@
     <t>keluar</t>
   </si>
   <si>
-    <t>KT-vn7ymgja</t>
+    <t>KT-qn7csaai</t>
   </si>
   <si>
     <t>Transportasi</t>
   </si>
   <si>
-    <t>KT-zypqn64g</t>
+    <t>KT-a2biljhn</t>
   </si>
   <si>
     <t>Belanja</t>
   </si>
   <si>
-    <t>KT-kd3hpnwa</t>
+    <t>KT-bp7ssihl</t>
   </si>
   <si>
     <t>Tagihan</t>
   </si>
   <si>
-    <t>KT-jyj4aba4</t>
+    <t>KT-xr3r52rp</t>
   </si>
   <si>
     <t>Pulsa &amp; Internet</t>
   </si>
   <si>
-    <t>KT-5hhpmopp</t>
+    <t>KT-6spivybc</t>
   </si>
   <si>
     <t>Langganan</t>
   </si>
   <si>
-    <t>KT-rjup5g53</t>
+    <t>KT-qk77lxlf</t>
   </si>
   <si>
     <t>Hiburan</t>
   </si>
   <si>
-    <t>KT-rxyf3wmq</t>
+    <t>KT-gzaymfuf</t>
   </si>
   <si>
     <t>Kesehatan</t>
   </si>
   <si>
-    <t>KT-afar6zpe</t>
+    <t>KT-ofitmcmo</t>
   </si>
   <si>
     <t>Pendidikan</t>
   </si>
   <si>
-    <t>KT-aibtphmp</t>
+    <t>KT-obatcyoh</t>
   </si>
   <si>
     <t>Sedekah</t>
   </si>
   <si>
-    <t>KT-3ixkre6q</t>
+    <t>KT-rlmchiet</t>
   </si>
   <si>
     <t>Biaya Admin Bank</t>
@@ -958,10 +1003,7 @@
     <t>BIAYA_ADMIN</t>
   </si>
   <si>
-    <t>KT-wyyzlhl3</t>
-  </si>
-  <si>
-    <t>user_id</t>
+    <t>KT-cju4cyg2</t>
   </si>
   <si>
     <t>tanggal_mulai</t>
@@ -974,9 +1016,6 @@
   </si>
   <si>
     <t>periode_id</t>
-  </si>
-  <si>
-    <t>akun_id</t>
   </si>
   <si>
     <t>saldo</t>
@@ -1589,6 +1628,346 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H50"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="28" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="28" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+    </row>
+    <row r="3" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+    </row>
+    <row r="4" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+    </row>
+    <row r="5" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+    </row>
+    <row r="6" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+    </row>
+    <row r="7" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+    </row>
+    <row r="8" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+    </row>
+    <row r="9" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+    </row>
+    <row r="10" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+    </row>
+    <row r="11" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
+    </row>
+    <row r="12" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+    </row>
+    <row r="13" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+    </row>
+    <row r="14" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
+    </row>
+    <row r="15" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6"/>
+    </row>
+    <row r="16" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+    </row>
+    <row r="17" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="6"/>
+    </row>
+    <row r="18" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6"/>
+      <c r="H18" s="6"/>
+    </row>
+    <row r="19" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+    </row>
+    <row r="20" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="6"/>
+    </row>
+    <row r="21" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+    </row>
+    <row r="22" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
+      <c r="G22" s="6"/>
+      <c r="H22" s="6"/>
+    </row>
+    <row r="23" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+    </row>
+    <row r="24" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
+    </row>
+    <row r="25" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="6"/>
+      <c r="H25" s="6"/>
+    </row>
+    <row r="26" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="6"/>
+      <c r="H26" s="6"/>
+    </row>
+    <row r="27" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="6"/>
+    </row>
+    <row r="28" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E28" s="6"/>
+      <c r="F28" s="6"/>
+      <c r="G28" s="6"/>
+      <c r="H28" s="6"/>
+    </row>
+    <row r="29" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E29" s="6"/>
+      <c r="F29" s="6"/>
+      <c r="G29" s="6"/>
+      <c r="H29" s="6"/>
+    </row>
+    <row r="30" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E30" s="6"/>
+      <c r="F30" s="6"/>
+      <c r="G30" s="6"/>
+      <c r="H30" s="6"/>
+    </row>
+    <row r="31" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E31" s="6"/>
+      <c r="F31" s="6"/>
+      <c r="G31" s="6"/>
+      <c r="H31" s="6"/>
+    </row>
+    <row r="32" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E32" s="6"/>
+      <c r="F32" s="6"/>
+      <c r="G32" s="6"/>
+      <c r="H32" s="6"/>
+    </row>
+    <row r="33" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E33" s="6"/>
+      <c r="F33" s="6"/>
+      <c r="G33" s="6"/>
+      <c r="H33" s="6"/>
+    </row>
+    <row r="34" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E34" s="6"/>
+      <c r="F34" s="6"/>
+      <c r="G34" s="6"/>
+      <c r="H34" s="6"/>
+    </row>
+    <row r="35" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E35" s="6"/>
+      <c r="F35" s="6"/>
+      <c r="G35" s="6"/>
+      <c r="H35" s="6"/>
+    </row>
+    <row r="36" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E36" s="6"/>
+      <c r="F36" s="6"/>
+      <c r="G36" s="6"/>
+      <c r="H36" s="6"/>
+    </row>
+    <row r="37" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
+    </row>
+    <row r="38" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E38" s="6"/>
+      <c r="F38" s="6"/>
+      <c r="G38" s="6"/>
+      <c r="H38" s="6"/>
+    </row>
+    <row r="39" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E39" s="6"/>
+      <c r="F39" s="6"/>
+      <c r="G39" s="6"/>
+      <c r="H39" s="6"/>
+    </row>
+    <row r="40" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E40" s="6"/>
+      <c r="F40" s="6"/>
+      <c r="G40" s="6"/>
+      <c r="H40" s="6"/>
+    </row>
+    <row r="41" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E41" s="6"/>
+      <c r="F41" s="6"/>
+      <c r="G41" s="6"/>
+      <c r="H41" s="6"/>
+    </row>
+    <row r="42" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E42" s="6"/>
+      <c r="F42" s="6"/>
+      <c r="G42" s="6"/>
+      <c r="H42" s="6"/>
+    </row>
+    <row r="43" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E43" s="6"/>
+      <c r="F43" s="6"/>
+      <c r="G43" s="6"/>
+      <c r="H43" s="6"/>
+    </row>
+    <row r="44" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E44" s="6"/>
+      <c r="F44" s="6"/>
+      <c r="G44" s="6"/>
+      <c r="H44" s="6"/>
+    </row>
+    <row r="45" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E45" s="6"/>
+      <c r="F45" s="6"/>
+      <c r="G45" s="6"/>
+      <c r="H45" s="6"/>
+    </row>
+    <row r="46" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E46" s="6"/>
+      <c r="F46" s="6"/>
+      <c r="G46" s="6"/>
+      <c r="H46" s="6"/>
+    </row>
+    <row r="47" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E47" s="6"/>
+      <c r="F47" s="6"/>
+      <c r="G47" s="6"/>
+      <c r="H47" s="6"/>
+    </row>
+    <row r="48" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E48" s="6"/>
+      <c r="F48" s="6"/>
+      <c r="G48" s="6"/>
+      <c r="H48" s="6"/>
+    </row>
+    <row r="49" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E49" s="6"/>
+      <c r="F49" s="6"/>
+      <c r="G49" s="6"/>
+      <c r="H49" s="6"/>
+    </row>
+    <row r="50" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E50" s="6"/>
+      <c r="F50" s="6"/>
+      <c r="G50" s="6"/>
+      <c r="H50" s="6"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:M50"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -1607,7 +1986,7 @@
         <v>20</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>94</v>
+        <v>51</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>101</v>
@@ -1616,16 +1995,16 @@
         <v>34</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>99</v>
+        <v>52</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>104</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="I1" s="4" t="s">
         <v>113</v>
@@ -2782,6 +3161,346 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H50"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="28" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="28" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+    </row>
+    <row r="3" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+    </row>
+    <row r="4" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+    </row>
+    <row r="5" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+    </row>
+    <row r="6" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+    </row>
+    <row r="7" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+    </row>
+    <row r="8" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+    </row>
+    <row r="9" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+    </row>
+    <row r="10" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+    </row>
+    <row r="11" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
+    </row>
+    <row r="12" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+    </row>
+    <row r="13" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+    </row>
+    <row r="14" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
+    </row>
+    <row r="15" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6"/>
+    </row>
+    <row r="16" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+    </row>
+    <row r="17" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="6"/>
+    </row>
+    <row r="18" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6"/>
+      <c r="H18" s="6"/>
+    </row>
+    <row r="19" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+    </row>
+    <row r="20" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="6"/>
+    </row>
+    <row r="21" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+    </row>
+    <row r="22" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
+      <c r="G22" s="6"/>
+      <c r="H22" s="6"/>
+    </row>
+    <row r="23" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+    </row>
+    <row r="24" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
+    </row>
+    <row r="25" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="6"/>
+      <c r="H25" s="6"/>
+    </row>
+    <row r="26" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="6"/>
+      <c r="H26" s="6"/>
+    </row>
+    <row r="27" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="6"/>
+    </row>
+    <row r="28" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E28" s="6"/>
+      <c r="F28" s="6"/>
+      <c r="G28" s="6"/>
+      <c r="H28" s="6"/>
+    </row>
+    <row r="29" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E29" s="6"/>
+      <c r="F29" s="6"/>
+      <c r="G29" s="6"/>
+      <c r="H29" s="6"/>
+    </row>
+    <row r="30" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E30" s="6"/>
+      <c r="F30" s="6"/>
+      <c r="G30" s="6"/>
+      <c r="H30" s="6"/>
+    </row>
+    <row r="31" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E31" s="6"/>
+      <c r="F31" s="6"/>
+      <c r="G31" s="6"/>
+      <c r="H31" s="6"/>
+    </row>
+    <row r="32" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E32" s="6"/>
+      <c r="F32" s="6"/>
+      <c r="G32" s="6"/>
+      <c r="H32" s="6"/>
+    </row>
+    <row r="33" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E33" s="6"/>
+      <c r="F33" s="6"/>
+      <c r="G33" s="6"/>
+      <c r="H33" s="6"/>
+    </row>
+    <row r="34" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E34" s="6"/>
+      <c r="F34" s="6"/>
+      <c r="G34" s="6"/>
+      <c r="H34" s="6"/>
+    </row>
+    <row r="35" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E35" s="6"/>
+      <c r="F35" s="6"/>
+      <c r="G35" s="6"/>
+      <c r="H35" s="6"/>
+    </row>
+    <row r="36" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E36" s="6"/>
+      <c r="F36" s="6"/>
+      <c r="G36" s="6"/>
+      <c r="H36" s="6"/>
+    </row>
+    <row r="37" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
+    </row>
+    <row r="38" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E38" s="6"/>
+      <c r="F38" s="6"/>
+      <c r="G38" s="6"/>
+      <c r="H38" s="6"/>
+    </row>
+    <row r="39" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E39" s="6"/>
+      <c r="F39" s="6"/>
+      <c r="G39" s="6"/>
+      <c r="H39" s="6"/>
+    </row>
+    <row r="40" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E40" s="6"/>
+      <c r="F40" s="6"/>
+      <c r="G40" s="6"/>
+      <c r="H40" s="6"/>
+    </row>
+    <row r="41" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E41" s="6"/>
+      <c r="F41" s="6"/>
+      <c r="G41" s="6"/>
+      <c r="H41" s="6"/>
+    </row>
+    <row r="42" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E42" s="6"/>
+      <c r="F42" s="6"/>
+      <c r="G42" s="6"/>
+      <c r="H42" s="6"/>
+    </row>
+    <row r="43" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E43" s="6"/>
+      <c r="F43" s="6"/>
+      <c r="G43" s="6"/>
+      <c r="H43" s="6"/>
+    </row>
+    <row r="44" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E44" s="6"/>
+      <c r="F44" s="6"/>
+      <c r="G44" s="6"/>
+      <c r="H44" s="6"/>
+    </row>
+    <row r="45" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E45" s="6"/>
+      <c r="F45" s="6"/>
+      <c r="G45" s="6"/>
+      <c r="H45" s="6"/>
+    </row>
+    <row r="46" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E46" s="6"/>
+      <c r="F46" s="6"/>
+      <c r="G46" s="6"/>
+      <c r="H46" s="6"/>
+    </row>
+    <row r="47" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E47" s="6"/>
+      <c r="F47" s="6"/>
+      <c r="G47" s="6"/>
+      <c r="H47" s="6"/>
+    </row>
+    <row r="48" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E48" s="6"/>
+      <c r="F48" s="6"/>
+      <c r="G48" s="6"/>
+      <c r="H48" s="6"/>
+    </row>
+    <row r="49" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E49" s="6"/>
+      <c r="F49" s="6"/>
+      <c r="G49" s="6"/>
+      <c r="H49" s="6"/>
+    </row>
+    <row r="50" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E50" s="6"/>
+      <c r="F50" s="6"/>
+      <c r="G50" s="6"/>
+      <c r="H50" s="6"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I50"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -2801,10 +3520,10 @@
         <v>23</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>25</v>
@@ -2824,13 +3543,13 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D2" t="s">
         <v>2</v>
@@ -2853,13 +3572,13 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" t="s">
         <v>57</v>
-      </c>
-      <c r="C3" t="s">
-        <v>55</v>
       </c>
       <c r="D3" t="s">
         <v>2</v>
@@ -2882,13 +3601,13 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D4" t="s">
         <v>2</v>
@@ -2911,13 +3630,13 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D5" t="s">
         <v>2</v>
@@ -2940,13 +3659,13 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B6" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D6" t="s">
         <v>2</v>
@@ -2969,13 +3688,13 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B7" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C7" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D7" t="s">
         <v>2</v>
@@ -2998,16 +3717,16 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E8" t="b">
         <v>1</v>
@@ -3027,13 +3746,13 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B9" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D9" t="s">
         <v>2</v>
@@ -3056,13 +3775,13 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B10" t="s">
+        <v>75</v>
+      </c>
+      <c r="C10" t="s">
         <v>73</v>
-      </c>
-      <c r="C10" t="s">
-        <v>71</v>
       </c>
       <c r="D10" t="s">
         <v>2</v>
@@ -3085,13 +3804,13 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B11" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D11" t="s">
         <v>2</v>
@@ -3114,13 +3833,13 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B12" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D12" t="s">
         <v>2</v>
@@ -3143,13 +3862,13 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B13" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D13" t="s">
         <v>2</v>
@@ -3172,13 +3891,13 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B14" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C14" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D14" t="s">
         <v>2</v>
@@ -3201,13 +3920,13 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B15" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D15" t="s">
         <v>2</v>
@@ -3230,13 +3949,13 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B16" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C16" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D16" t="s">
         <v>2</v>
@@ -3259,13 +3978,13 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B17" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C17" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D17" t="s">
         <v>2</v>
@@ -3288,13 +4007,13 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D18" t="s">
         <v>2</v>
@@ -3317,16 +4036,16 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B19" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C19" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D19" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E19" t="b">
         <v>1</v>
@@ -3346,13 +4065,13 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C20" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D20" t="s">
         <v>2</v>
@@ -3568,7 +4287,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J50"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -3587,19 +4306,19 @@
         <v>20</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>94</v>
+        <v>51</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>23</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>30</v>
@@ -3915,7 +4634,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I50"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -3933,13 +4652,13 @@
         <v>20</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>94</v>
+        <v>51</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>99</v>
+        <v>52</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>100</v>
@@ -4258,7 +4977,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:P50"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -4281,19 +5000,19 @@
         <v>20</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>94</v>
+        <v>51</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>101</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>99</v>
+        <v>52</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>102</v>
@@ -4632,7 +5351,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:O50"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -4653,13 +5372,13 @@
         <v>20</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>94</v>
+        <v>51</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>23</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>99</v>
+        <v>52</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>103</v>
@@ -4988,346 +5707,6 @@
       <c r="M50" s="6"/>
       <c r="N50" s="6"/>
       <c r="O50" s="6"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <legacyDrawing r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H50"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="28" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="28" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-    </row>
-    <row r="3" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-    </row>
-    <row r="4" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-    </row>
-    <row r="5" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-    </row>
-    <row r="6" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-    </row>
-    <row r="7" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-    </row>
-    <row r="8" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
-    </row>
-    <row r="9" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-    </row>
-    <row r="10" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-    </row>
-    <row r="11" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-    </row>
-    <row r="12" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-    </row>
-    <row r="13" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-    </row>
-    <row r="14" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-    </row>
-    <row r="15" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-    </row>
-    <row r="16" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
-    </row>
-    <row r="17" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="6"/>
-    </row>
-    <row r="18" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
-    </row>
-    <row r="19" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
-    </row>
-    <row r="20" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E20" s="6"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
-      <c r="H20" s="6"/>
-    </row>
-    <row r="21" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
-    </row>
-    <row r="22" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E22" s="6"/>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="6"/>
-    </row>
-    <row r="23" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
-    </row>
-    <row r="24" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
-      <c r="H24" s="6"/>
-    </row>
-    <row r="25" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E25" s="6"/>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
-      <c r="H25" s="6"/>
-    </row>
-    <row r="26" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
-      <c r="H26" s="6"/>
-    </row>
-    <row r="27" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E27" s="6"/>
-      <c r="F27" s="6"/>
-      <c r="G27" s="6"/>
-      <c r="H27" s="6"/>
-    </row>
-    <row r="28" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E28" s="6"/>
-      <c r="F28" s="6"/>
-      <c r="G28" s="6"/>
-      <c r="H28" s="6"/>
-    </row>
-    <row r="29" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E29" s="6"/>
-      <c r="F29" s="6"/>
-      <c r="G29" s="6"/>
-      <c r="H29" s="6"/>
-    </row>
-    <row r="30" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E30" s="6"/>
-      <c r="F30" s="6"/>
-      <c r="G30" s="6"/>
-      <c r="H30" s="6"/>
-    </row>
-    <row r="31" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E31" s="6"/>
-      <c r="F31" s="6"/>
-      <c r="G31" s="6"/>
-      <c r="H31" s="6"/>
-    </row>
-    <row r="32" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E32" s="6"/>
-      <c r="F32" s="6"/>
-      <c r="G32" s="6"/>
-      <c r="H32" s="6"/>
-    </row>
-    <row r="33" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E33" s="6"/>
-      <c r="F33" s="6"/>
-      <c r="G33" s="6"/>
-      <c r="H33" s="6"/>
-    </row>
-    <row r="34" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E34" s="6"/>
-      <c r="F34" s="6"/>
-      <c r="G34" s="6"/>
-      <c r="H34" s="6"/>
-    </row>
-    <row r="35" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E35" s="6"/>
-      <c r="F35" s="6"/>
-      <c r="G35" s="6"/>
-      <c r="H35" s="6"/>
-    </row>
-    <row r="36" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E36" s="6"/>
-      <c r="F36" s="6"/>
-      <c r="G36" s="6"/>
-      <c r="H36" s="6"/>
-    </row>
-    <row r="37" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E37" s="6"/>
-      <c r="F37" s="6"/>
-      <c r="G37" s="6"/>
-      <c r="H37" s="6"/>
-    </row>
-    <row r="38" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E38" s="6"/>
-      <c r="F38" s="6"/>
-      <c r="G38" s="6"/>
-      <c r="H38" s="6"/>
-    </row>
-    <row r="39" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E39" s="6"/>
-      <c r="F39" s="6"/>
-      <c r="G39" s="6"/>
-      <c r="H39" s="6"/>
-    </row>
-    <row r="40" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E40" s="6"/>
-      <c r="F40" s="6"/>
-      <c r="G40" s="6"/>
-      <c r="H40" s="6"/>
-    </row>
-    <row r="41" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E41" s="6"/>
-      <c r="F41" s="6"/>
-      <c r="G41" s="6"/>
-      <c r="H41" s="6"/>
-    </row>
-    <row r="42" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E42" s="6"/>
-      <c r="F42" s="6"/>
-      <c r="G42" s="6"/>
-      <c r="H42" s="6"/>
-    </row>
-    <row r="43" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E43" s="6"/>
-      <c r="F43" s="6"/>
-      <c r="G43" s="6"/>
-      <c r="H43" s="6"/>
-    </row>
-    <row r="44" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E44" s="6"/>
-      <c r="F44" s="6"/>
-      <c r="G44" s="6"/>
-      <c r="H44" s="6"/>
-    </row>
-    <row r="45" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E45" s="6"/>
-      <c r="F45" s="6"/>
-      <c r="G45" s="6"/>
-      <c r="H45" s="6"/>
-    </row>
-    <row r="46" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E46" s="6"/>
-      <c r="F46" s="6"/>
-      <c r="G46" s="6"/>
-      <c r="H46" s="6"/>
-    </row>
-    <row r="47" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E47" s="6"/>
-      <c r="F47" s="6"/>
-      <c r="G47" s="6"/>
-      <c r="H47" s="6"/>
-    </row>
-    <row r="48" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E48" s="6"/>
-      <c r="F48" s="6"/>
-      <c r="G48" s="6"/>
-      <c r="H48" s="6"/>
-    </row>
-    <row r="49" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E49" s="6"/>
-      <c r="F49" s="6"/>
-      <c r="G49" s="6"/>
-      <c r="H49" s="6"/>
-    </row>
-    <row r="50" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E50" s="6"/>
-      <c r="F50" s="6"/>
-      <c r="G50" s="6"/>
-      <c r="H50" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>